<commit_message>
added women3 generated pictures and data for clip model
</commit_message>
<xml_diff>
--- a/Models/CLIP/female1data/clip_big5_female1_no_makeup.xlsx
+++ b/Models/CLIP/female1data/clip_big5_female1_no_makeup.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="23" documentId="11_C796E7C9C49E9A8A7A47FBBA53B94F015B504C7B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5416733D-8E6B-4726-A77E-7485E3C888CC}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9760" windowHeight="11370" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extraversion" sheetId="1" r:id="rId1"/>
@@ -229,7 +229,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>